<commit_message>
Second commit. 5-6 phases
</commit_message>
<xml_diff>
--- a/Reestr_proektnyh_dokumentov_v.0.2.xlsx
+++ b/Reestr_proektnyh_dokumentov_v.0.2.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\YandexDisk\Проектное управление (шаблоны документов)\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\YandexDisk\Проектное управление (шаблоны документов)\Project documents (samples)\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A87EA3CA-BCCB-46B0-8545-DB6A2775B3D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D625065-A2A0-4BE2-92D2-C7E3EE4B2D3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3630" yWindow="4350" windowWidth="25860" windowHeight="16530" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="16410" yWindow="1695" windowWidth="25860" windowHeight="16530" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Инструкция" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="243">
   <si>
     <t>РЕЕСТР ПРОЕКТНЫХ ДОКУМЕНТОВ</t>
   </si>
@@ -743,6 +743,33 @@
   </si>
   <si>
     <t>Protokol_kod-revyu_shablon.docx</t>
+  </si>
+  <si>
+    <t>Plan_podderzhki_Hypercare_shablon.docx</t>
+  </si>
+  <si>
+    <t>Zhurnal_zamechaniy_OPE.xlsx</t>
+  </si>
+  <si>
+    <t>Reglament_OPE_shablon.docx</t>
+  </si>
+  <si>
+    <t>Plan_obucheniya_shablon.docx</t>
+  </si>
+  <si>
+    <t>Detalnyy_plan_migracii_shablon.docx</t>
+  </si>
+  <si>
+    <t>Plan_razvyortyvaniya_Cutover_shablon.docx</t>
+  </si>
+  <si>
+    <t>Zhurnal_defektov.xlsx</t>
+  </si>
+  <si>
+    <t>Protokol_priyomochnyh_ispytaniy_shablon.docx</t>
+  </si>
+  <si>
+    <t>Protokol_testirovaniya_shablon.docx</t>
   </si>
 </sst>
 </file>
@@ -2496,9 +2523,11 @@
         <v>39</v>
       </c>
       <c r="E46" s="13" t="s">
-        <v>86</v>
-      </c>
-      <c r="F46" s="13"/>
+        <v>33</v>
+      </c>
+      <c r="F46" s="13" t="s">
+        <v>242</v>
+      </c>
       <c r="G46" s="13" t="s">
         <v>151</v>
       </c>
@@ -2520,9 +2549,11 @@
         <v>51</v>
       </c>
       <c r="E47" s="13" t="s">
-        <v>86</v>
-      </c>
-      <c r="F47" s="13"/>
+        <v>33</v>
+      </c>
+      <c r="F47" s="13" t="s">
+        <v>240</v>
+      </c>
       <c r="G47" s="13" t="s">
         <v>151</v>
       </c>
@@ -2544,9 +2575,11 @@
         <v>39</v>
       </c>
       <c r="E48" s="13" t="s">
-        <v>86</v>
-      </c>
-      <c r="F48" s="13"/>
+        <v>33</v>
+      </c>
+      <c r="F48" s="13" t="s">
+        <v>241</v>
+      </c>
       <c r="G48" s="13" t="s">
         <v>151</v>
       </c>
@@ -2580,9 +2613,11 @@
         <v>39</v>
       </c>
       <c r="E50" s="13" t="s">
-        <v>86</v>
-      </c>
-      <c r="F50" s="13"/>
+        <v>33</v>
+      </c>
+      <c r="F50" s="13" t="s">
+        <v>239</v>
+      </c>
       <c r="G50" s="13" t="s">
         <v>164</v>
       </c>
@@ -2604,9 +2639,11 @@
         <v>39</v>
       </c>
       <c r="E51" s="13" t="s">
-        <v>86</v>
-      </c>
-      <c r="F51" s="13"/>
+        <v>33</v>
+      </c>
+      <c r="F51" s="13" t="s">
+        <v>238</v>
+      </c>
       <c r="G51" s="13" t="s">
         <v>125</v>
       </c>
@@ -2628,9 +2665,11 @@
         <v>39</v>
       </c>
       <c r="E52" s="13" t="s">
-        <v>86</v>
-      </c>
-      <c r="F52" s="13"/>
+        <v>33</v>
+      </c>
+      <c r="F52" s="13" t="s">
+        <v>237</v>
+      </c>
       <c r="G52" s="13" t="s">
         <v>169</v>
       </c>
@@ -2652,9 +2691,11 @@
         <v>39</v>
       </c>
       <c r="E53" s="13" t="s">
-        <v>86</v>
-      </c>
-      <c r="F53" s="13"/>
+        <v>33</v>
+      </c>
+      <c r="F53" s="13" t="s">
+        <v>236</v>
+      </c>
       <c r="G53" s="13" t="s">
         <v>41</v>
       </c>
@@ -2676,9 +2717,11 @@
         <v>51</v>
       </c>
       <c r="E54" s="13" t="s">
-        <v>86</v>
-      </c>
-      <c r="F54" s="13"/>
+        <v>33</v>
+      </c>
+      <c r="F54" s="13" t="s">
+        <v>235</v>
+      </c>
       <c r="G54" s="13" t="s">
         <v>41</v>
       </c>
@@ -2700,9 +2743,11 @@
         <v>39</v>
       </c>
       <c r="E55" s="13" t="s">
-        <v>86</v>
-      </c>
-      <c r="F55" s="13"/>
+        <v>33</v>
+      </c>
+      <c r="F55" s="13" t="s">
+        <v>234</v>
+      </c>
       <c r="G55" s="13" t="s">
         <v>41</v>
       </c>
@@ -3019,7 +3064,7 @@
       </c>
       <c r="C7" s="16">
         <f>COUNTIF('Реестр документов'!$E$3:$E$65,"Готов")</f>
-        <v>38</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8" spans="2:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3037,7 +3082,7 @@
       </c>
       <c r="C9" s="16">
         <f>COUNTIF('Реестр документов'!$E$3:$E$65,"Не создан")</f>
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10" spans="2:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3064,7 +3109,7 @@
       </c>
       <c r="C12" s="22">
         <f>IFERROR(COUNTIF('Реестр документов'!$E$3:$E$65,"Готов")/(COUNTIF('Реестр документов'!$E$3:$E$65,"Готов")+COUNTIF('Реестр документов'!$E$3:$E$65,"В работе")+COUNTIF('Реестр документов'!$E$3:$E$65,"Не создан")),0)</f>
-        <v>0.69090909090909092</v>
+        <v>0.8545454545454545</v>
       </c>
     </row>
     <row r="14" spans="2:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>